<commit_message>
fix(boiling): pass historical-data integration acceptance
</commit_message>
<xml_diff>
--- a/modules/boiling/tests/fixtures/samples/actual/demo_run/boiling_summary.xlsx
+++ b/modules/boiling/tests/fixtures/samples/actual/demo_run/boiling_summary.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水煮检测汇总" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="试件明细" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规则说明" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分析图表" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="水煮检测汇总" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="未纳入正常统计" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="试件明细" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="规则说明" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="分析图表" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'水煮检测汇总'!$A$1:$S$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'试件明细'!$A$1:$Q$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'水煮检测汇总'!$A$1:$AE$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'未纳入正常统计'!$A$1:$H$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'试件明细'!$A$1:$V$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +27,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,8 +40,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <name val="微软雅黑"/>
+      <color rgb="00000000"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -49,6 +55,26 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -69,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -80,7 +106,19 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -160,13 +198,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -190,7 +228,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -230,8 +268,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -255,13 +293,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -285,7 +323,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -325,8 +363,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -350,7 +388,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -365,9 +403,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -387,9 +425,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -687,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S8"/>
+  <dimension ref="A1:AE8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -695,20 +733,32 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="44" customWidth="1" min="17" max="17"/>
-    <col width="28" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="50" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="48" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="30" customWidth="1" min="25" max="25"/>
+    <col width="34" customWidth="1" min="26" max="26"/>
+    <col width="26" customWidth="1" min="27" max="27"/>
+    <col width="26" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="16" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -779,32 +829,92 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>最小密度(g/cm³)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>最大密度(g/cm³)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>密度差(g/cm³)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>密度规则</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>平均膨胀率</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>膨胀率规则</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>自动等级</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>需人工复核</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>浸渍剥离</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>原表结论</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>缺失字段</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>业务状态</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>缺失/待补字段</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>命中规则ID</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>密度来源单元格</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>膨胀率来源单元格</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>复算冲突数</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>结论/规则冲突数</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>源表有效区域</t>
         </is>
       </c>
     </row>
@@ -869,24 +979,78 @@
         <v>1.2</v>
       </c>
       <c r="N2" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O2" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="P2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="O2" s="4" t="n">
+      <c r="Q2" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="R2" s="5" t="n">
         <v>0.05000000000000006</v>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>膨胀率≤6.5%，需结合开裂观察确认绿色优等</t>
+        </is>
+      </c>
+      <c r="T2" s="4" t="inlineStr">
+        <is>
+          <t>绿色优等候选</t>
+        </is>
+      </c>
+      <c r="U2" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
         <is>
           <t>合格</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>密度检测合格，2h膨胀率检测合格，浸渍剥离检测合格 检测员 脱敏测试员</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="inlineStr"/>
-      <c r="S2" s="2" t="n">
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>密度检测合格，2h膨胀率检测合格，浸渍剥离检测合格</t>
+        </is>
+      </c>
+      <c r="X2" s="4" t="inlineStr">
+        <is>
+          <t>正常</t>
+        </is>
+      </c>
+      <c r="Y2" s="2" t="inlineStr"/>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>BOILING-DENSITY-001, BOILING-EXPANSION-001</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>F12, F19</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>H12, H19</t>
+        </is>
+      </c>
+      <c r="AC2" s="2" t="n">
         <v>0</v>
+      </c>
+      <c r="AD2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="2" t="inlineStr">
+        <is>
+          <t>A1:H23</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -950,24 +1114,78 @@
         <v>1.45</v>
       </c>
       <c r="N3" s="3" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="P3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="O3" s="4" t="n">
+      <c r="Q3" s="7" t="inlineStr">
+        <is>
+          <t>不合格</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="n">
         <v>0.05000000000000006</v>
       </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>膨胀率≤6.5%，需结合开裂观察确认绿色优等</t>
+        </is>
+      </c>
+      <c r="T3" s="4" t="inlineStr">
+        <is>
+          <t>绿色优等候选</t>
+        </is>
+      </c>
+      <c r="U3" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
         <is>
           <t>合格</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>密度检测待复核，2h膨胀率检测合格，浸渍剥离检测合格 检测员 脱敏测试员</t>
-        </is>
-      </c>
-      <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="n">
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>密度检测待复核，2h膨胀率检测合格，浸渍剥离检测合格</t>
+        </is>
+      </c>
+      <c r="X3" s="6" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr">
+        <is>
+          <t>BOILING-DENSITY-001, BOILING-EXPANSION-001</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
+          <t>F12, F19</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>H12, H19</t>
+        </is>
+      </c>
+      <c r="AC3" s="2" t="n">
         <v>0</v>
+      </c>
+      <c r="AD3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE3" s="2" t="inlineStr">
+        <is>
+          <t>A1:H23</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -1031,24 +1249,78 @@
         <v>1.2</v>
       </c>
       <c r="N4" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="P4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="n">
         <v>0.1</v>
       </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>膨胀率＞8%，红色不合格</t>
+        </is>
+      </c>
+      <c r="T4" s="7" t="inlineStr">
+        <is>
+          <t>红色不合格</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="inlineStr">
         <is>
           <t>合格</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="inlineStr">
-        <is>
-          <t>密度检测合格，2h膨胀率检测待复核，浸渍剥离检测合格 检测员 脱敏测试员</t>
-        </is>
-      </c>
-      <c r="R4" s="2" t="inlineStr"/>
-      <c r="S4" s="2" t="n">
+      <c r="W4" s="2" t="inlineStr">
+        <is>
+          <t>密度检测合格，2h膨胀率检测待复核，浸渍剥离检测合格</t>
+        </is>
+      </c>
+      <c r="X4" s="6" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr">
+        <is>
+          <t>BOILING-DENSITY-001, BOILING-EXPANSION-001</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
+          <t>F12, F19</t>
+        </is>
+      </c>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>H12, H19</t>
+        </is>
+      </c>
+      <c r="AC4" s="2" t="n">
         <v>0</v>
+      </c>
+      <c r="AD4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE4" s="2" t="inlineStr">
+        <is>
+          <t>A1:H23</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -1112,24 +1384,78 @@
         <v>1.2</v>
       </c>
       <c r="N5" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="P5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="O5" s="4" t="n">
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="R5" s="5" t="n">
         <v>0.05000000000000006</v>
       </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>膨胀率≤6.5%，需结合开裂观察确认绿色优等</t>
+        </is>
+      </c>
+      <c r="T5" s="4" t="inlineStr">
+        <is>
+          <t>绿色优等候选</t>
+        </is>
+      </c>
+      <c r="U5" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="V5" s="2" t="inlineStr">
         <is>
           <t>不合格</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="inlineStr">
-        <is>
-          <t>密度检测合格，2h膨胀率检测合格，浸渍剥离检测不合格 检测员 脱敏测试员</t>
-        </is>
-      </c>
-      <c r="R5" s="2" t="inlineStr"/>
-      <c r="S5" s="2" t="n">
+      <c r="W5" s="2" t="inlineStr">
+        <is>
+          <t>密度检测合格，2h膨胀率检测合格，浸渍剥离检测不合格</t>
+        </is>
+      </c>
+      <c r="X5" s="7" t="inlineStr">
+        <is>
+          <t>异常</t>
+        </is>
+      </c>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>BOILING-DENSITY-001, BOILING-EXPANSION-001</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="inlineStr">
+        <is>
+          <t>F12, F19</t>
+        </is>
+      </c>
+      <c r="AB5" s="2" t="inlineStr">
+        <is>
+          <t>H12, H19</t>
+        </is>
+      </c>
+      <c r="AC5" s="2" t="n">
         <v>0</v>
+      </c>
+      <c r="AD5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>A1:H23</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -1193,24 +1519,78 @@
         <v>1.2</v>
       </c>
       <c r="N6" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="P6" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="O6" s="4" t="n">
+      <c r="Q6" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="n">
         <v>0.05000000000000007</v>
       </c>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>膨胀率≤6.5%，需结合开裂观察确认绿色优等</t>
+        </is>
+      </c>
+      <c r="T6" s="4" t="inlineStr">
+        <is>
+          <t>绿色优等候选</t>
+        </is>
+      </c>
+      <c r="U6" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="inlineStr">
         <is>
           <t>合格</t>
         </is>
       </c>
-      <c r="Q6" s="2" t="inlineStr">
-        <is>
-          <t>复测完成，浸渍剥离检测合格 检测员 脱敏测试员</t>
-        </is>
-      </c>
-      <c r="R6" s="2" t="inlineStr"/>
-      <c r="S6" s="2" t="n">
+      <c r="W6" s="2" t="inlineStr">
+        <is>
+          <t>复测完成，浸渍剥离检测合格</t>
+        </is>
+      </c>
+      <c r="X6" s="4" t="inlineStr">
+        <is>
+          <t>正常</t>
+        </is>
+      </c>
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr">
+        <is>
+          <t>BOILING-DENSITY-001, BOILING-EXPANSION-001</t>
+        </is>
+      </c>
+      <c r="AA6" s="2" t="inlineStr">
+        <is>
+          <t>F12, F19, F26</t>
+        </is>
+      </c>
+      <c r="AB6" s="2" t="inlineStr">
+        <is>
+          <t>H12, H19, H26</t>
+        </is>
+      </c>
+      <c r="AC6" s="2" t="n">
         <v>0</v>
+      </c>
+      <c r="AD6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="2" t="inlineStr">
+        <is>
+          <t>A1:H30</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -1274,24 +1654,78 @@
         <v>1.18</v>
       </c>
       <c r="N7" s="3" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="P7" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="O7" s="4" t="n">
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="n">
         <v>0.04000000000000003</v>
       </c>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>膨胀率≤6.5%，需结合开裂观察确认绿色优等</t>
+        </is>
+      </c>
+      <c r="T7" s="4" t="inlineStr">
+        <is>
+          <t>绿色优等候选</t>
+        </is>
+      </c>
+      <c r="U7" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr">
         <is>
           <t>合格</t>
         </is>
       </c>
-      <c r="Q7" s="2" t="inlineStr">
-        <is>
-          <t>密度检测合格，2h膨胀率检测合格，浸渍剥离检测合格 检测员 脱敏测试员</t>
-        </is>
-      </c>
-      <c r="R7" s="2" t="inlineStr"/>
-      <c r="S7" s="2" t="n">
+      <c r="W7" s="2" t="inlineStr">
+        <is>
+          <t>密度检测合格，2h膨胀率检测合格，浸渍剥离检测合格</t>
+        </is>
+      </c>
+      <c r="X7" s="4" t="inlineStr">
+        <is>
+          <t>正常</t>
+        </is>
+      </c>
+      <c r="Y7" s="2" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr">
+        <is>
+          <t>BOILING-DENSITY-001, BOILING-EXPANSION-001</t>
+        </is>
+      </c>
+      <c r="AA7" s="2" t="inlineStr">
+        <is>
+          <t>F12, F19, F26</t>
+        </is>
+      </c>
+      <c r="AB7" s="2" t="inlineStr">
+        <is>
+          <t>H12, H19, H26</t>
+        </is>
+      </c>
+      <c r="AC7" s="2" t="n">
         <v>0</v>
+      </c>
+      <c r="AD7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="2" t="inlineStr">
+        <is>
+          <t>A1:H30</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -1355,28 +1789,82 @@
         <v>1.2</v>
       </c>
       <c r="N8" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="P8" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="O8" s="4" t="n">
+      <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="S8" s="2" t="inlineStr">
+        <is>
+          <t>膨胀率≤6.5%，需结合开裂观察确认绿色优等</t>
+        </is>
+      </c>
+      <c r="T8" s="4" t="inlineStr">
+        <is>
+          <t>绿色优等候选</t>
+        </is>
+      </c>
+      <c r="U8" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="V8" s="2" t="inlineStr">
         <is>
           <t>合格</t>
         </is>
       </c>
-      <c r="Q8" s="2" t="inlineStr">
-        <is>
-          <t>密度检测合格，2h膨胀率检测合格，浸渍剥离检测合格 检测员 脱敏测试员</t>
-        </is>
-      </c>
-      <c r="R8" s="2" t="inlineStr"/>
-      <c r="S8" s="2" t="n">
+      <c r="W8" s="2" t="inlineStr">
+        <is>
+          <t>密度检测合格，2h膨胀率检测合格，浸渍剥离检测合格</t>
+        </is>
+      </c>
+      <c r="X8" s="6" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y8" s="2" t="inlineStr"/>
+      <c r="Z8" s="2" t="inlineStr">
+        <is>
+          <t>BOILING-DENSITY-001, BOILING-EXPANSION-001</t>
+        </is>
+      </c>
+      <c r="AA8" s="2" t="inlineStr">
+        <is>
+          <t>F12</t>
+        </is>
+      </c>
+      <c r="AB8" s="2" t="inlineStr">
+        <is>
+          <t>H12</t>
+        </is>
+      </c>
+      <c r="AC8" s="2" t="n">
         <v>2</v>
       </c>
+      <c r="AD8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="2" t="inlineStr">
+        <is>
+          <t>A1:H16</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S8"/>
+  <autoFilter ref="A1:AE8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1387,7 +1875,116 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="54" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>来源文件</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>批号</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>产品</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>规格</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>业务状态</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>缺失字段</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>阻断原因</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>处理说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>07_empty_incomplete.xlsx</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>DEMO-007</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>规格型号</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>版本</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>信息不足</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>source_conclusion</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>未识别到测量试件；原表标记为未完成</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>空表、未完成表或无可计算试件；未进入正常汇总和图表统计。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1398,12 +1995,17 @@
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1464,30 +2066,55 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>原表显示密度</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>复算密度</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>采用密度</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>密度规则</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>密度来源单元格</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>原表膨胀率</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>原表显示膨胀率</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>复算膨胀率</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>采用膨胀率</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>膨胀率来源单元格</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>来源区域</t>
         </is>
@@ -1535,22 +2162,47 @@
       <c r="K2" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="L2" s="3" t="n">
-        <v>1.2</v>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>1.200</t>
+        </is>
       </c>
       <c r="M2" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="N2" s="4" t="n">
+      <c r="N2" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>F12</t>
+        </is>
+      </c>
+      <c r="Q2" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="O2" s="4" t="n">
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="P2" s="4" t="n">
+      <c r="T2" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>H12</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
         <is>
           <t>A6:H12</t>
         </is>
@@ -1598,24 +2250,49 @@
       <c r="K3" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="L3" s="3" t="n">
-        <v>1.2</v>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>1.200</t>
+        </is>
       </c>
       <c r="M3" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="N3" s="4" t="n">
+      <c r="N3" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="O3" s="4" t="n">
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="n">
         <v>0.05000000000000012</v>
       </c>
-      <c r="P3" s="4" t="n">
+      <c r="T3" s="5" t="n">
         <v>0.05000000000000012</v>
       </c>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>A13:H19</t>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>H19</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>A13:H20</t>
         </is>
       </c>
     </row>
@@ -1661,22 +2338,47 @@
       <c r="K4" s="3" t="n">
         <v>1.45</v>
       </c>
-      <c r="L4" s="3" t="n">
-        <v>1.45</v>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>1.450</t>
+        </is>
       </c>
       <c r="M4" s="3" t="n">
         <v>1.45</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="N4" s="3" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="O4" s="7" t="inlineStr">
+        <is>
+          <t>不合格</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>F12</t>
+        </is>
+      </c>
+      <c r="Q4" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="S4" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="T4" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="Q4" s="2" t="inlineStr">
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>H12</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="inlineStr">
         <is>
           <t>A6:H12</t>
         </is>
@@ -1724,24 +2426,49 @@
       <c r="K5" s="3" t="n">
         <v>1.45</v>
       </c>
-      <c r="L5" s="3" t="n">
-        <v>1.45</v>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>1.450</t>
+        </is>
       </c>
       <c r="M5" s="3" t="n">
         <v>1.45</v>
       </c>
-      <c r="N5" s="4" t="n">
+      <c r="N5" s="3" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="O5" s="7" t="inlineStr">
+        <is>
+          <t>不合格</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="O5" s="4" t="n">
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="S5" s="5" t="n">
         <v>0.05000000000000012</v>
       </c>
-      <c r="P5" s="4" t="n">
+      <c r="T5" s="5" t="n">
         <v>0.05000000000000012</v>
       </c>
-      <c r="Q5" s="2" t="inlineStr">
-        <is>
-          <t>A13:H19</t>
+      <c r="U5" s="2" t="inlineStr">
+        <is>
+          <t>H19</t>
+        </is>
+      </c>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>A13:H20</t>
         </is>
       </c>
     </row>
@@ -1787,22 +2514,47 @@
       <c r="K6" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="L6" s="3" t="n">
-        <v>1.2</v>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>1.200</t>
+        </is>
       </c>
       <c r="M6" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="N6" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>F12</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="n">
         <v>0.1</v>
       </c>
-      <c r="O6" s="4" t="n">
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="S6" s="5" t="n">
         <v>0.1</v>
       </c>
-      <c r="P6" s="4" t="n">
+      <c r="T6" s="5" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q6" s="2" t="inlineStr">
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>H12</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="inlineStr">
         <is>
           <t>A6:H12</t>
         </is>
@@ -1850,24 +2602,49 @@
       <c r="K7" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="L7" s="3" t="n">
-        <v>1.2</v>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>1.200</t>
+        </is>
       </c>
       <c r="M7" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="N7" s="4" t="n">
+      <c r="N7" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="n">
         <v>0.1</v>
       </c>
-      <c r="O7" s="4" t="n">
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="S7" s="5" t="n">
         <v>0.1000000000000001</v>
       </c>
-      <c r="P7" s="4" t="n">
+      <c r="T7" s="5" t="n">
         <v>0.1000000000000001</v>
       </c>
-      <c r="Q7" s="2" t="inlineStr">
-        <is>
-          <t>A13:H19</t>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>H19</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>A13:H20</t>
         </is>
       </c>
     </row>
@@ -1913,22 +2690,47 @@
       <c r="K8" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="L8" s="3" t="n">
-        <v>1.2</v>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>1.200</t>
+        </is>
       </c>
       <c r="M8" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="N8" s="4" t="n">
+      <c r="N8" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>F12</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="O8" s="4" t="n">
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="P8" s="4" t="n">
+      <c r="T8" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="Q8" s="2" t="inlineStr">
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>H12</t>
+        </is>
+      </c>
+      <c r="V8" s="2" t="inlineStr">
         <is>
           <t>A6:H12</t>
         </is>
@@ -1976,24 +2778,49 @@
       <c r="K9" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="L9" s="3" t="n">
-        <v>1.2</v>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>1.200</t>
+        </is>
       </c>
       <c r="M9" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="N9" s="4" t="n">
+      <c r="N9" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="O9" s="4" t="n">
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="S9" s="5" t="n">
         <v>0.05000000000000012</v>
       </c>
-      <c r="P9" s="4" t="n">
+      <c r="T9" s="5" t="n">
         <v>0.05000000000000012</v>
       </c>
-      <c r="Q9" s="2" t="inlineStr">
-        <is>
-          <t>A13:H19</t>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>H19</t>
+        </is>
+      </c>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>A13:H20</t>
         </is>
       </c>
     </row>
@@ -2039,22 +2866,47 @@
       <c r="K10" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="L10" s="3" t="n">
-        <v>1.2</v>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>1.200</t>
+        </is>
       </c>
       <c r="M10" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="N10" s="4" t="n">
+      <c r="N10" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>F12</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="O10" s="4" t="n">
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="S10" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="P10" s="4" t="n">
+      <c r="T10" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="Q10" s="2" t="inlineStr">
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>H12</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
         <is>
           <t>A6:H12</t>
         </is>
@@ -2102,22 +2954,47 @@
       <c r="K11" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="L11" s="3" t="n">
-        <v>1.2</v>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>1.200</t>
+        </is>
       </c>
       <c r="M11" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="N11" s="4" t="n">
+      <c r="N11" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="O11" s="4" t="n">
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="n">
         <v>0.05000000000000012</v>
       </c>
-      <c r="P11" s="4" t="n">
+      <c r="T11" s="5" t="n">
         <v>0.05000000000000012</v>
       </c>
-      <c r="Q11" s="2" t="inlineStr">
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>H19</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
         <is>
           <t>A13:H19</t>
         </is>
@@ -2165,24 +3042,49 @@
       <c r="K12" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="L12" s="3" t="n">
-        <v>1.2</v>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>1.200</t>
+        </is>
       </c>
       <c r="M12" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="N12" s="4" t="n">
+      <c r="N12" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>F26</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="O12" s="4" t="n">
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="n">
         <v>0.05000000000000007</v>
       </c>
-      <c r="P12" s="4" t="n">
+      <c r="T12" s="5" t="n">
         <v>0.05000000000000007</v>
       </c>
-      <c r="Q12" s="2" t="inlineStr">
-        <is>
-          <t>A20:H26</t>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>H26</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>A20:H27</t>
         </is>
       </c>
     </row>
@@ -2228,22 +3130,47 @@
       <c r="K13" s="3" t="n">
         <v>1.18</v>
       </c>
-      <c r="L13" s="3" t="n">
-        <v>1.18</v>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>1.180</t>
+        </is>
       </c>
       <c r="M13" s="3" t="n">
         <v>1.18</v>
       </c>
-      <c r="N13" s="4" t="n">
+      <c r="N13" s="3" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>F12</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="n">
         <v>0.04</v>
       </c>
-      <c r="O13" s="4" t="n">
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>4.00%</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="n">
         <v>0.04000000000000004</v>
       </c>
-      <c r="P13" s="4" t="n">
+      <c r="T13" s="5" t="n">
         <v>0.04000000000000004</v>
       </c>
-      <c r="Q13" s="2" t="inlineStr">
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>H12</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
         <is>
           <t>A6:H12</t>
         </is>
@@ -2291,22 +3218,47 @@
       <c r="K14" s="3" t="n">
         <v>1.18</v>
       </c>
-      <c r="L14" s="3" t="n">
-        <v>1.18</v>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>1.180</t>
+        </is>
       </c>
       <c r="M14" s="3" t="n">
         <v>1.18</v>
       </c>
-      <c r="N14" s="4" t="n">
+      <c r="N14" s="3" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="n">
         <v>0.04</v>
       </c>
-      <c r="O14" s="4" t="n">
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>4.00%</t>
+        </is>
+      </c>
+      <c r="S14" s="5" t="n">
         <v>0.04000000000000003</v>
       </c>
-      <c r="P14" s="4" t="n">
+      <c r="T14" s="5" t="n">
         <v>0.04000000000000003</v>
       </c>
-      <c r="Q14" s="2" t="inlineStr">
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>H19</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
         <is>
           <t>A13:H19</t>
         </is>
@@ -2354,24 +3306,49 @@
       <c r="K15" s="3" t="n">
         <v>1.18</v>
       </c>
-      <c r="L15" s="3" t="n">
-        <v>1.18</v>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>1.180</t>
+        </is>
       </c>
       <c r="M15" s="3" t="n">
         <v>1.18</v>
       </c>
-      <c r="N15" s="4" t="n">
+      <c r="N15" s="3" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>F26</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="n">
         <v>0.04</v>
       </c>
-      <c r="O15" s="4" t="n">
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>4.00%</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="n">
         <v>0.04000000000000002</v>
       </c>
-      <c r="P15" s="4" t="n">
+      <c r="T15" s="5" t="n">
         <v>0.04000000000000002</v>
       </c>
-      <c r="Q15" s="2" t="inlineStr">
-        <is>
-          <t>A20:H26</t>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>H26</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>A20:H27</t>
         </is>
       </c>
     </row>
@@ -2417,40 +3394,65 @@
       <c r="K16" s="3" t="n">
         <v>1.28</v>
       </c>
-      <c r="L16" s="3" t="n">
-        <v>1.2</v>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>1.280</t>
+        </is>
       </c>
       <c r="M16" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="N16" s="4" t="n">
+      <c r="N16" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
+          <t>合格</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>F12</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="n">
         <v>0.08</v>
       </c>
-      <c r="O16" s="4" t="n">
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>8.00%</t>
+        </is>
+      </c>
+      <c r="S16" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="P16" s="4" t="n">
+      <c r="T16" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="Q16" s="2" t="inlineStr">
-        <is>
-          <t>A6:H12</t>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>H12</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>A6:H13</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q16"/>
+  <autoFilter ref="A1:V16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2465,7 +3467,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>2026.07-draft</t>
+          <t>2026.07.18-v0.1</t>
         </is>
       </c>
     </row>
@@ -2477,43 +3479,79 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>pending_customer_confirmation</t>
+          <t>confirmed_with_wall_railing_review_gap</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>重要说明</t>
+          <t>密度正式规则</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>客户未确认的阈值仅用于异常观察，不生成正式合格/不合格结论。</t>
+          <t>每个有效试件 1.1～1.3 g/cm³（含边界），且最大值-最小值≤0.1 g/cm³（含边界）。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>密度暂存范围</t>
+          <t>绿色优等</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1.1 ~ 1.3 g/cm³</t>
+          <t>平均膨胀率≤6.5%，并须结合表面、侧面和端头开裂观察人工确认。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>膨胀率规则</t>
+          <t>地板/家具</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>必须先确定产品用途，再按用途选择阈值；未知用途转人工确认。</t>
+          <t>6.5%＜平均膨胀率≤8% 为蓝色合格；＞8% 为红色不合格。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>墙板/栏杆</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>8%≤平均膨胀率≤12% 为蓝色合格；＞12% 为红色不合格。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>v0.1 人工边界</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>墙板/栏杆平均膨胀率＞6.5%且＜8% 不自动标色，转人工复核。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>用途缺失</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>不得猜测产品用途；生成一次可批量应用的确认项。</t>
         </is>
       </c>
     </row>
@@ -2522,7 +3560,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2562,7 +3600,7 @@
       <c r="B2" s="2" t="n">
         <v>1.2</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="5" t="n">
         <v>0.05000000000000006</v>
       </c>
     </row>
@@ -2575,7 +3613,7 @@
       <c r="B3" s="2" t="n">
         <v>1.45</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="5" t="n">
         <v>0.05000000000000006</v>
       </c>
     </row>
@@ -2588,7 +3626,7 @@
       <c r="B4" s="2" t="n">
         <v>1.2</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="5" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -2601,7 +3639,7 @@
       <c r="B5" s="2" t="n">
         <v>1.2</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="5" t="n">
         <v>0.05000000000000006</v>
       </c>
     </row>
@@ -2614,7 +3652,7 @@
       <c r="B6" s="2" t="n">
         <v>1.2</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="5" t="n">
         <v>0.05000000000000007</v>
       </c>
     </row>
@@ -2627,7 +3665,7 @@
       <c r="B7" s="2" t="n">
         <v>1.18</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="5" t="n">
         <v>0.04000000000000003</v>
       </c>
     </row>
@@ -2640,7 +3678,7 @@
       <c r="B8" s="2" t="n">
         <v>1.2</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="5" t="n">
         <v>0.05</v>
       </c>
     </row>

</xml_diff>